<commit_message>
Release v1.3.0 catalog publishing
</commit_message>
<xml_diff>
--- a/assets/Card-Sale-Manager-Import-Template.xlsx
+++ b/assets/Card-Sale-Manager-Import-Template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Card Import" sheetId="1" r:id="R59338cc60bb44d8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Card Import" sheetId="1" r:id="R483674cf070e427e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,12 +13,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
+  <x:numFmts count="4">
     <x:numFmt numFmtId="200" formatCode="0"/>
     <x:numFmt numFmtId="201" formatCode="@"/>
     <x:numFmt numFmtId="202" formatCode="&quot;$&quot;#,##0.00"/>
+    <x:numFmt numFmtId="203" formatCode="$#,##0.00"/>
   </x:numFmts>
-  <x:fonts count="3">
+  <x:fonts count="4">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -33,6 +34,12 @@
       <x:sz val="10"/>
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
   <x:fills count="5">
@@ -159,7 +166,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="60">
+  <x:cellXfs count="66">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -335,12 +342,49 @@
     </x:xf>
     <x:xf numFmtId="201" fontId="1" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CardImportTable" displayName="CardImportTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="11">
+    <x:tableColumn id="1" name="Year"/>
+    <x:tableColumn id="2" name="Brand"/>
+    <x:tableColumn id="3" name="Player"/>
+    <x:tableColumn id="4" name="Number"/>
+    <x:tableColumn id="5" name="Sport"/>
+    <x:tableColumn id="6" name="Team(s)"/>
+    <x:tableColumn id="7" name="Flaw(s)"/>
+    <x:tableColumn id="8" name="Grade"/>
+    <x:tableColumn id="9" name="Claim Price"/>
+    <x:tableColumn id="10" name="Purchase Price"/>
+    <x:tableColumn id="11" name="Purchase Date"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -542,14 +586,16 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="11" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="15" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="15" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="17" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -566,18 +612,24 @@
         <x:v>Number</x:v>
       </x:c>
       <x:c r="E1" s="6" t="str">
+        <x:v>Sport</x:v>
+      </x:c>
+      <x:c r="F1" s="6" t="str">
+        <x:v>Team(s)</x:v>
+      </x:c>
+      <x:c r="G1" s="6" t="str">
         <x:v>Flaw(s)</x:v>
       </x:c>
-      <x:c r="F1" s="6" t="str">
+      <x:c r="H1" s="6" t="str">
         <x:v>Grade</x:v>
       </x:c>
-      <x:c r="G1" s="6" t="str">
+      <x:c r="I1" s="6" t="str">
         <x:v>Claim Price</x:v>
       </x:c>
-      <x:c r="H1" s="6" t="str">
+      <x:c r="J1" s="61" t="str">
         <x:v>Purchase Price</x:v>
       </x:c>
-      <x:c r="I1" s="6" t="str">
+      <x:c r="K1" s="61" t="str">
         <x:v>Purchase Date</x:v>
       </x:c>
     </x:row>
@@ -595,18 +647,24 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="E2" s="32" t="str">
+        <x:v>Baseball</x:v>
+      </x:c>
+      <x:c r="F2" s="48" t="str">
+        <x:v>Los Angeles Dodgers</x:v>
+      </x:c>
+      <x:c r="G2" s="52" t="str">
         <x:v>Clean back</x:v>
       </x:c>
-      <x:c r="F2" s="48" t="str">
+      <x:c r="H2" s="52" t="str">
         <x:v>VG-EX</x:v>
       </x:c>
-      <x:c r="G2" s="52" t="n">
+      <x:c r="I2" s="62" t="n">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="H2" s="52" t="n">
+      <x:c r="J2" s="63" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="I2" s="56" t="str">
+      <x:c r="K2" s="65" t="str">
         <x:v>09172026</x:v>
       </x:c>
     </x:row>
@@ -624,18 +682,24 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="E3" s="33" t="str">
+        <x:v>Baseball</x:v>
+      </x:c>
+      <x:c r="F3" s="49" t="str">
+        <x:v>New York Yankees; Los Angeles Dodgers</x:v>
+      </x:c>
+      <x:c r="G3" s="53" t="str">
         <x:v>Soft corners</x:v>
       </x:c>
-      <x:c r="F3" s="49" t="str">
+      <x:c r="H3" s="53" t="str">
         <x:v>VG</x:v>
       </x:c>
-      <x:c r="G3" s="53" t="n">
+      <x:c r="I3" s="64" t="n">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="H3" s="53" t="n">
+      <x:c r="J3" s="63" t="n">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="I3" s="57" t="str">
+      <x:c r="K3" s="65" t="str">
         <x:v>09172026</x:v>
       </x:c>
     </x:row>
@@ -653,18 +717,24 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="E4" s="33" t="str">
+        <x:v>Baseball</x:v>
+      </x:c>
+      <x:c r="F4" s="49" t="str">
+        <x:v>St. Louis Cardinals</x:v>
+      </x:c>
+      <x:c r="G4" s="53" t="str">
         <x:v>None</x:v>
       </x:c>
-      <x:c r="F4" s="49" t="str">
+      <x:c r="H4" s="53" t="str">
         <x:v>EX</x:v>
       </x:c>
-      <x:c r="G4" s="53" t="n">
+      <x:c r="I4" s="64" t="n">
         <x:v>59</x:v>
       </x:c>
-      <x:c r="H4" s="53" t="n">
+      <x:c r="J4" s="63" t="n">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="I4" s="57" t="str">
+      <x:c r="K4" s="65" t="str">
         <x:v>09172026</x:v>
       </x:c>
     </x:row>
@@ -1769,7 +1839,7 @@
       <x:c r="I104" s="59"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="2">
+  <x:dataValidations count="3">
     <x:dataValidation type="whole" operator="between" sqref="A2:A104">
       <x:formula1>1800</x:formula1>
       <x:formula2>2100</x:formula2>
@@ -1777,7 +1847,13 @@
     <x:dataValidation type="decimal" operator="greaterThanOrEqual" sqref="G2:H104">
       <x:formula1>0</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="E2:E500">
+      <x:formula1>"Baseball,Basketball,Football,Hockey,Other"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra135e68bede44ec9"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>